<commit_message>
some what working code mostly
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/INPUTS/classrooms-template.xlsx
+++ b/TIME TABLE SAMPLE DATA/INPUTS/classrooms-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5afc8f5c19c83632/Desktop/Timetable/TIME TABLE SAMPLE DATA/INPUTS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="11_2B59D2BFD3C0546BF9ADABD34C3088B352998D1A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3FD786E-92E3-46D3-8728-1A9DA1D5D720}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="11_2B59D2BFD3C0546BF9ADABD34C3088B352998D1A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{015BD1E9-B268-44AA-A721-A78D4660DE70}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -729,7 +729,7 @@
         <v>2</v>
       </c>
       <c r="C15">
-        <v>75</v>
+        <v>3175</v>
       </c>
       <c r="D15" t="s">
         <v>20</v>

</xml_diff>